<commit_message>
Prepare Student Tracker for rollout: versioned release build, startup hardening, docs
Co-Authored-By: Gillam TCMed <ccp71044@gmail.com>
</commit_message>
<xml_diff>
--- a/Student Tracker.xlsx
+++ b/Student Tracker.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\agill\Dropbox\Allens Training\Courses\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6684B817-58E9-44A0-8ACF-00DD0555F0C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39FDFBB4-0971-47D0-BFAF-D9BAB1F7B863}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{38A4FFF0-5798-4AE8-B957-35DB0DFA192A}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="120">
   <si>
     <t>Student Register</t>
   </si>
@@ -387,6 +387,18 @@
   </si>
   <si>
     <t>Stacey</t>
+  </si>
+  <si>
+    <t>AG</t>
+  </si>
+  <si>
+    <t>Ag</t>
+  </si>
+  <si>
+    <t>HLTPAT010</t>
+  </si>
+  <si>
+    <t>FTO</t>
   </si>
 </sst>
 </file>
@@ -488,7 +500,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -526,9 +538,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -865,7 +874,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8DC0EBF-7BDB-4CC1-8DD3-14D0E6409807}">
-  <dimension ref="A1:P45"/>
+  <dimension ref="A1:P47"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.140625" customWidth="1"/>
@@ -891,7 +900,7 @@
       </c>
       <c r="K1">
         <f>SUM(G3:G9999)</f>
-        <v>1358</v>
+        <v>1498</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
@@ -924,7 +933,7 @@
       </c>
       <c r="K2">
         <f>O25-K1</f>
-        <v>46</v>
+        <v>-94</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
@@ -1686,7 +1695,7 @@
       <c r="A39" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="B39" s="14" t="s">
+      <c r="B39" s="12" t="s">
         <v>109</v>
       </c>
       <c r="G39">
@@ -1697,11 +1706,17 @@
       </c>
     </row>
     <row r="40" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A40" s="14" t="s">
-        <v>110</v>
-      </c>
-      <c r="B40" s="14" t="s">
-        <v>111</v>
+      <c r="A40" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="B40" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="E40" t="s">
+        <v>16</v>
+      </c>
+      <c r="F40" s="1">
+        <v>46256</v>
       </c>
       <c r="G40">
         <v>20</v>
@@ -1711,10 +1726,10 @@
       </c>
     </row>
     <row r="41" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A41" s="14" t="s">
+      <c r="A41" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="B41" s="14" t="s">
+      <c r="B41" s="12" t="s">
         <v>111</v>
       </c>
       <c r="G41">
@@ -1725,7 +1740,7 @@
       </c>
     </row>
     <row r="42" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A42" s="14" t="s">
+      <c r="A42" s="12" t="s">
         <v>112</v>
       </c>
       <c r="G42">
@@ -1733,7 +1748,7 @@
       </c>
     </row>
     <row r="43" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A43" s="14" t="s">
+      <c r="A43" s="12" t="s">
         <v>113</v>
       </c>
       <c r="G43">
@@ -1741,7 +1756,7 @@
       </c>
     </row>
     <row r="44" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A44" s="14" t="s">
+      <c r="A44" s="12" t="s">
         <v>114</v>
       </c>
       <c r="G44">
@@ -1749,11 +1764,33 @@
       </c>
     </row>
     <row r="45" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A45" s="14" t="s">
+      <c r="A45" s="12" t="s">
         <v>115</v>
       </c>
       <c r="G45">
         <v>9</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A46" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="E46" t="s">
+        <v>118</v>
+      </c>
+      <c r="G46">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A47" s="12" t="s">
+        <v>117</v>
+      </c>
+      <c r="E47" t="s">
+        <v>119</v>
+      </c>
+      <c r="G47">
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>